<commit_message>
modified media storage url based on vercel blob
</commit_message>
<xml_diff>
--- a/media.xlsx
+++ b/media.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VENKAT\Downloads\LEARNING\my-podcasts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VENKAT\Downloads\LEARNING\media-podcasts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BBFF9E8-A4FE-4707-BA9C-5BB2AEB5B2A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3264CB-99A7-4703-84EC-9B6783F396D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,9 +45,6 @@
     <t>Data Science Introduction</t>
   </si>
   <si>
-    <t>Data_Science_Toolkit.mp4</t>
-  </si>
-  <si>
     <t>Tech.</t>
   </si>
   <si>
@@ -57,37 +54,40 @@
     <t>audio</t>
   </si>
   <si>
-    <t>Jimmy_the_scarlet_sailor.mp4</t>
-  </si>
-  <si>
-    <t>Jimmy_the_scarlet_sailor.m4a</t>
-  </si>
-  <si>
     <t>Story</t>
   </si>
   <si>
     <t>The Algorithm of Courage</t>
   </si>
   <si>
-    <t>The_algorithm_of_courage.m4a</t>
-  </si>
-  <si>
     <t>The Bosphorus Bluff</t>
   </si>
   <si>
-    <t>The_Bosphorus_Bluff.m4a</t>
-  </si>
-  <si>
-    <t>The_illusion_of_creation.m4a</t>
-  </si>
-  <si>
     <t>The Illusion of Creation</t>
   </si>
   <si>
-    <t>डर_के_आगे_जीत_है.m4a</t>
-  </si>
-  <si>
     <t>डर_के_आगे_जीत_है</t>
+  </si>
+  <si>
+    <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/Data_Science_Toolkit.mp4</t>
+  </si>
+  <si>
+    <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/Jimmy_the_Scarlet_Sailor.mp4</t>
+  </si>
+  <si>
+    <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/Jimmy_the_scarlet%20_sailor.m4a</t>
+  </si>
+  <si>
+    <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/The_Bosphorus_Bluff.m4a</t>
+  </si>
+  <si>
+    <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/The_algorithm_of_courage.m4a</t>
+  </si>
+  <si>
+    <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/The_illusion_of_creation.m4a</t>
+  </si>
+  <si>
+    <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/%E0%A4%A1%E0%A4%B0_%E0%A4%95%E0%A5%87_%E0%A4%86%E0%A4%97%E0%A5%87_%E0%A4%9C%E0%A5%80%E0%A4%A4_%E0%A4%B9%E0%A5%88.m4a</t>
   </si>
 </sst>
 </file>
@@ -415,7 +415,7 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.46484375" customWidth="1"/>
-    <col min="3" max="3" width="27.265625" customWidth="1"/>
+    <col min="3" max="3" width="180.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
@@ -440,94 +440,94 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
         <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
         <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
         <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
         <v>20</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
         <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added another podcast maritime ai pilot purgatory
</commit_message>
<xml_diff>
--- a/media.xlsx
+++ b/media.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VENKAT\Downloads\LEARNING\media-podcasts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3264CB-99A7-4703-84EC-9B6783F396D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D190A2B-4806-4063-BAFC-4261A484265B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
   <si>
     <t>title</t>
   </si>
@@ -88,13 +88,19 @@
   </si>
   <si>
     <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/%E0%A4%A1%E0%A4%B0_%E0%A4%95%E0%A5%87_%E0%A4%86%E0%A4%97%E0%A5%87_%E0%A4%9C%E0%A5%80%E0%A4%A4_%E0%A4%B9%E0%A5%88.m4a</t>
+  </si>
+  <si>
+    <t>Maritime AI in Pilot Purgatory</t>
+  </si>
+  <si>
+    <t>https://wavphq1kc6ulbtnz.public.blob.vercel-storage.com/Maritime_AI_in_Pilot_Purgatory.m4a</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -104,6 +110,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -126,13 +140,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -411,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.46484375" customWidth="1"/>
@@ -530,8 +547,25 @@
         <v>9</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C9" r:id="rId1" xr:uid="{1344E455-2583-4F4D-937F-FAB686139A5F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>